<commit_message>
Lots of changes to improve output.
Made sure years were integers, added ability to hide teaching evals.  Reformatted $ amounts
</commit_message>
<xml_diff>
--- a/src/make_cv/files/Awards/personal awards data.xlsx
+++ b/src/make_cv/files/Awards/personal awards data.xlsx
@@ -1,48 +1,91 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bhelenbr/Codes/make_cv/src/make_cv/files/Awards/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E179135F-9338-B84F-B742-88390270AC20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4440" yWindow="760" windowWidth="25800" windowHeight="17300" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="4440" yWindow="720" windowWidth="25800" windowHeight="17300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notes" sheetId="1" r:id="rId1"/>
+    <sheet name="Data" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+  <si>
+    <t>This sheet is to keep track of awards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Make an entry in data for every award </t>
+  </si>
+  <si>
+    <t>Types:</t>
+  </si>
+  <si>
+    <t>Professional</t>
+  </si>
+  <si>
+    <t>School</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>University</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Excellence in Teaching</t>
+  </si>
+  <si>
+    <t>Best Paper Award at USNCCM</t>
+  </si>
+  <si>
+    <t>Examples</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="12"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="8"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -61,12 +104,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -96,75 +139,75 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1" tint="0.499984740745262"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1" tint="0.499984740745262"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="0" tint="-0.1499984740745262"/>
-          <bgColor theme="0" tint="-0.1499984740745262"/>
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
         </patternFill>
       </fill>
       <border>
         <left style="thin">
-          <color theme="0" tint="-0.3499862666707358"/>
+          <color theme="0" tint="-0.34998626667073579"/>
         </left>
         <right style="thin">
-          <color theme="0" tint="-0.3499862666707358"/>
+          <color theme="0" tint="-0.34998626667073579"/>
         </right>
         <top style="thin">
-          <color theme="0" tint="-0.3499862666707358"/>
+          <color theme="0" tint="-0.34998626667073579"/>
         </top>
         <bottom style="thin">
-          <color theme="0" tint="-0.3499862666707358"/>
+          <color theme="0" tint="-0.34998626667073579"/>
         </bottom>
         <vertical style="thin">
-          <color theme="0" tint="-0.3499862666707358"/>
+          <color theme="0" tint="-0.34998626667073579"/>
         </vertical>
         <horizontal style="thin">
-          <color theme="0" tint="-0.3499862666707358"/>
+          <color theme="0" tint="-0.34998626667073579"/>
         </horizontal>
       </border>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="0" tint="-0.1499984740745262"/>
-          <bgColor theme="0" tint="-0.1499984740745262"/>
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
         </patternFill>
       </fill>
       <border>
         <top style="thin">
-          <color theme="0" tint="-0.3499862666707358"/>
+          <color theme="0" tint="-0.34998626667073579"/>
         </top>
         <bottom style="thin">
-          <color theme="0" tint="-0.3499862666707358"/>
+          <color theme="0" tint="-0.34998626667073579"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
       <fill>
@@ -184,7 +227,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
       <border>
@@ -211,7 +254,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="PivotStyleLight1 2" table="0" count="11">
+    <tableStyle name="PivotStyleLight1 2" table="0" count="11" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="10"/>
       <tableStyleElement type="headerRow" dxfId="9"/>
       <tableStyleElement type="totalRow" dxfId="8"/>
@@ -225,74 +268,14 @@
       <tableStyleElement type="pageFieldValues" dxfId="0"/>
     </tableStyle>
   </tableStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -592,61 +575,84 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="26.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>This sheet is to keep track of awards</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Make an entry in data for every award </t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Types:</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Professional</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>School</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Department</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>University</t>
-        </is>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19">
+        <v>2025</v>
       </c>
     </row>
   </sheetData>
@@ -655,46 +661,45 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="22" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="22" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col width="30.5" customWidth="1" style="2" min="1" max="1"/>
-    <col width="15.6640625" customWidth="1" min="2" max="2"/>
-    <col width="12.6640625" customWidth="1" min="3" max="3"/>
+    <col min="1" max="1" width="30.5" style="2" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
+    <row r="1" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>Notes!$A$10:$A$13</formula1>
-    </dataValidation>
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="whole" operator="between">
+  <dataValidations count="1">
+    <dataValidation type="whole" sqref="C2:C1048576" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>1900</formula1>
       <formula2>2100</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000000000000}">
+          <x14:formula1>
+            <xm:f>Notes!$A$10:$A$13</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>